<commit_message>
R05 (em andamento): tabelas do artigo em .docx no formato pedido, números-chave, T13 e T15
- tabelas: A4, margens de 2,5 cm, Times New Roman 8, bordas de 0,5 pt, larguras pelo conteúdo;
  Painel B reproduz o artigo (T13); geração determinística (T15)
- números-chave com parâmetros, diagnóstico e checagens; tabelas também em ponto decimal
  (resultados/rodada05/tabelas_artigo_ponto_decimal.md) para o relatório
- simulações: registro do SOL por TWh sem a D18 (aba d18_SOL)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CWPuQS1EQNnCbSqHfPPCuA
</commit_message>
<xml_diff>
--- a/artigo/tabelas/tabelas_artigo.xlsx
+++ b/artigo/tabelas/tabelas_artigo.xlsx
@@ -2563,7 +2563,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Parcela da transmissão paga pela geração (α)</t>
+          <t>Parcela da transmissão paga pelo consumo, via distribuição (α); a geração paga 1 − α</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -2573,7 +2573,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Rateio inicial de 50% para a geração (ANEEL, REN nº 559/2013)</t>
+          <t>Rateio inicial dos encargos de uso: 50% geração e 50% consumo (ANEEL, REN nº 559/2013)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">

</xml_diff>

<commit_message>
R05 (em andamento): correções da revisão dos textos (Quadro 2, reprodução do artigo, alertas na B.12 e na Tabela A8, limitações 1 e 6, E2, Eq. 28, citações com ano entre colchetes) e relatório
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CWPuQS1EQNnCbSqHfPPCuA
</commit_message>
<xml_diff>
--- a/artigo/tabelas/tabelas_artigo.xlsx
+++ b/artigo/tabelas/tabelas_artigo.xlsx
@@ -5301,7 +5301,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -5475,7 +5475,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Os nove cenários do artigo, rodados na MIP original, reproduzem os valores publicados</t>
+          <t>Os nove cenários do artigo, rodados na MIP original, reproduzem os valores de referência; arredondados a uma casa, os Painéis B das Tabelas 1, 3 e 4 (exceto a linha R4a da Tabela 4) e a Tabela A2 são idênticos aos publicados</t>
         </is>
       </c>
       <c r="C10" s="6" t="n">
@@ -5483,7 +5483,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>t CO₂e (maior diferença)</t>
+          <t>t CO₂e (maior diferença nas emissões totais)</t>
         </is>
       </c>
     </row>
@@ -5507,15 +5507,35 @@
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>Nota: 'Valor' é a maior diferença absoluta encontrada (ou a contagem indicada); tolerância de 10⁻⁶ nas igualdades.</t>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Alertas</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Sem falhas. Alertas registrados: multiplicador de produção acima de 2,2 em 9 das 9 especificações (na principal: geração a gás natural do RS; geração a derivados de petróleo do RS, latente; gás canalizado e outras utilidades do RS; geração a derivados de petróleo do RB); insumos não energéticos da geração a gás natural abaixo de 5% do VBP em 7 (todas, exceto κ = 0,60 e η = 0,05)</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>falhas</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Nota: 'Valor' é a maior diferença absoluta encontrada (ou a contagem indicada); tolerância de 10⁻⁶ nas igualdades.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>Fonte: Elaboração própria.</t>
         </is>

</xml_diff>

<commit_message>
R05: versão final (MIP v04) — correções da verificação final (E3 sem total preservado, três tipos de alerta, linha da Tabela 4 com o vetor da Tabela A1, tolerância da Tabela A8, figuras em 7 × 4,4 pol) e relatório completo
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CWPuQS1EQNnCbSqHfPPCuA
</commit_message>
<xml_diff>
--- a/artigo/tabelas/tabelas_artigo.xlsx
+++ b/artigo/tabelas/tabelas_artigo.xlsx
@@ -5475,7 +5475,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Os nove cenários do artigo, rodados na MIP original, reproduzem os valores de referência; arredondados a uma casa, os Painéis B das Tabelas 1, 3 e 4 (exceto a linha R4a da Tabela 4) e a Tabela A2 são idênticos aos publicados</t>
+          <t>Os nove cenários do artigo, rodados na MIP original, reproduzem os valores de referência, com duas casas decimais; arredondados a uma casa, os Painéis B das Tabelas 1, 3 e 4 e a Tabela A2 são idênticos aos publicados, exceto a linha da Tabela 4 calculada com o vetor da Tabela A1</t>
         </is>
       </c>
       <c r="C10" s="6" t="n">
@@ -5495,7 +5495,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>As 9 especificações (principal e 8 variantes) passam nas mesmas checagens; nas variantes E3 e E4 as emissões preservam só o total</t>
+          <t>As 9 especificações (principal e 8 variantes) passam nas mesmas checagens; na E3, as emissões do S38 deixam de reproduzir a base (diferem pelo resíduo), e na E4 só o total da economia é preservado (alerta)</t>
         </is>
       </c>
       <c r="C11" s="6" t="n">
@@ -5515,7 +5515,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Sem falhas. Alertas registrados: multiplicador de produção acima de 2,2 em 9 das 9 especificações (na principal: geração a gás natural do RS; geração a derivados de petróleo do RS, latente; gás canalizado e outras utilidades do RS; geração a derivados de petróleo do RB); insumos não energéticos da geração a gás natural abaixo de 5% do VBP em 7 (todas, exceto κ = 0,60 e η = 0,05)</t>
+          <t>Sem falhas. Alertas registrados: multiplicador de produção acima de 2,2 em 9 das 9 especificações (na principal: geração a gás natural do RS; geração a derivados de petróleo do RS, latente; gás canalizado e outras utilidades do RS; geração a derivados de petróleo do RB); insumos não energéticos da geração a gás natural abaixo de 5% do VBP em 7 (todas, exceto κ = 0,60 e η = 0,05); preservação das emissões na E3 e na E4 (linha anterior)</t>
         </is>
       </c>
       <c r="C12" s="6" t="n">
@@ -5530,7 +5530,7 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Nota: 'Valor' é a maior diferença absoluta encontrada (ou a contagem indicada); tolerância de 10⁻⁶ nas igualdades.</t>
+          <t>Nota: 'Valor' é a maior diferença absoluta encontrada (ou a contagem indicada); tolerância de 10⁻⁶ nas igualdades, salvo na reprodução do artigo, comparada com valores de referência de duas casas decimais (tolerância de 1 t CO₂e).</t>
         </is>
       </c>
     </row>

</xml_diff>